<commit_message>
Added the complete logic to account for G&C and Chris delta
Signed-off-by: Bhavya <bhavya_b@mit.edu>
</commit_message>
<xml_diff>
--- a/output_excel/Chris - G&C Comparison.xlsx
+++ b/output_excel/Chris - G&C Comparison.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mitprod.sharepoint.com/sites/TruckParkingCapstone_zdvvwb/Shared Documents/General/Truck Stop Finder 🚚⛽/4. Working Data Files/Traffic Files/Capstone_truck/Python Code/TruckParking/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mitprod.sharepoint.com/sites/TruckParkingCapstone_zdvvwb/Shared Documents/General/Truck Stop Finder 🚚⛽/4. Working Data Files/Traffic Files/Capstone_truck/Python Code/TruckParking/output_excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="112" documentId="11_30B9C0F20DACFF4D8A3BD604D62CCFD5CAA601C4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C46DC3ED-B9C3-460D-873F-7D3DD0445B7E}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="11_30B9C0F20DACFF4D8A3BD604D62CCFD5CAA601C4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F485A0A0-835C-4F52-B3BE-A65509B0ED6A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79052,6 +79052,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06520203-CDB0-4C4C-B268-5AFBB2D07120}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L247"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -79104,7 +79105,7 @@
         <v>4643</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3007</v>
       </c>
@@ -79145,7 +79146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2894</v>
       </c>
@@ -79186,7 +79187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>449</v>
       </c>
@@ -79227,7 +79228,7 @@
         <v>-148</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2402</v>
       </c>
@@ -79268,7 +79269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4193</v>
       </c>
@@ -79309,7 +79310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>782</v>
       </c>
@@ -79350,7 +79351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>1983</v>
       </c>
@@ -79391,7 +79392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>2552</v>
       </c>
@@ -79432,7 +79433,7 @@
         <v>-32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4006</v>
       </c>
@@ -79473,7 +79474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>3274</v>
       </c>
@@ -79514,7 +79515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2609</v>
       </c>
@@ -79555,7 +79556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>1675</v>
       </c>
@@ -79637,7 +79638,7 @@
         <v>-35</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>693</v>
       </c>
@@ -79678,7 +79679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>1286</v>
       </c>
@@ -79719,7 +79720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>3914</v>
       </c>
@@ -79760,7 +79761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>4162</v>
       </c>
@@ -79799,7 +79800,7 @@
         <v>-79</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>4558</v>
       </c>
@@ -79840,7 +79841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>1363</v>
       </c>
@@ -79881,7 +79882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>2074</v>
       </c>
@@ -79919,7 +79920,7 @@
         <v>-70</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>3931</v>
       </c>
@@ -79960,7 +79961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>1980</v>
       </c>
@@ -80001,7 +80002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>2028</v>
       </c>
@@ -80042,7 +80043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>4320</v>
       </c>
@@ -80083,7 +80084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>3404</v>
       </c>
@@ -80124,7 +80125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>4438</v>
       </c>
@@ -80165,7 +80166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>4031</v>
       </c>
@@ -80206,7 +80207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>866</v>
       </c>
@@ -80247,7 +80248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>122</v>
       </c>
@@ -80288,7 +80289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>1547</v>
       </c>
@@ -80329,7 +80330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>3430</v>
       </c>
@@ -80370,7 +80371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>2970</v>
       </c>
@@ -80411,7 +80412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>466</v>
       </c>
@@ -80452,7 +80453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>3703</v>
       </c>
@@ -80493,7 +80494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>4399</v>
       </c>
@@ -80534,7 +80535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>4225</v>
       </c>
@@ -80575,7 +80576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>2350</v>
       </c>
@@ -80616,7 +80617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>4222</v>
       </c>
@@ -80657,7 +80658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>487</v>
       </c>
@@ -80698,7 +80699,7 @@
         <v>-73</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>4064</v>
       </c>
@@ -80739,7 +80740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>3127</v>
       </c>
@@ -80780,7 +80781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>1236</v>
       </c>
@@ -80821,7 +80822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>3716</v>
       </c>
@@ -80862,7 +80863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>299</v>
       </c>
@@ -80903,7 +80904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>2238</v>
       </c>
@@ -80944,7 +80945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>2009</v>
       </c>
@@ -80985,7 +80986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>1236</v>
       </c>
@@ -81026,7 +81027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>3086</v>
       </c>
@@ -81067,7 +81068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>487</v>
       </c>
@@ -81106,7 +81107,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>4146</v>
       </c>
@@ -81147,7 +81148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>4070</v>
       </c>
@@ -81188,7 +81189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>3334</v>
       </c>
@@ -81229,7 +81230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>2490</v>
       </c>
@@ -81270,7 +81271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>1990</v>
       </c>
@@ -81311,7 +81312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>2201</v>
       </c>
@@ -81352,7 +81353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>4245</v>
       </c>
@@ -81393,7 +81394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>899</v>
       </c>
@@ -81434,7 +81435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>2289</v>
       </c>
@@ -81475,7 +81476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>1492</v>
       </c>
@@ -81516,7 +81517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>3598</v>
       </c>
@@ -81557,7 +81558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>3015</v>
       </c>
@@ -81598,7 +81599,7 @@
         <v>-111</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>3299</v>
       </c>
@@ -81639,7 +81640,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>1164</v>
       </c>
@@ -81680,7 +81681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>2682</v>
       </c>
@@ -81721,7 +81722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>1909</v>
       </c>
@@ -81762,7 +81763,7 @@
         <v>-93</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>3077</v>
       </c>
@@ -81803,7 +81804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>3970</v>
       </c>
@@ -81844,7 +81845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>3023</v>
       </c>
@@ -81885,7 +81886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>4371</v>
       </c>
@@ -81926,7 +81927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>1460</v>
       </c>
@@ -82008,7 +82009,7 @@
         <v>-86</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>2065</v>
       </c>
@@ -82049,7 +82050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>1236</v>
       </c>
@@ -82090,7 +82091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>1089</v>
       </c>
@@ -82131,7 +82132,7 @@
         <v>-47</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>4342</v>
       </c>
@@ -82172,7 +82173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>2703</v>
       </c>
@@ -82213,7 +82214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>1769</v>
       </c>
@@ -82254,7 +82255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>1236</v>
       </c>
@@ -82295,7 +82296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>3838</v>
       </c>
@@ -82336,7 +82337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>2626</v>
       </c>
@@ -82377,7 +82378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>1636</v>
       </c>
@@ -82418,7 +82419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>2638</v>
       </c>
@@ -82459,7 +82460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>835</v>
       </c>
@@ -82500,7 +82501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>494</v>
       </c>
@@ -82538,7 +82539,7 @@
         <v>-50</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>1091</v>
       </c>
@@ -82579,7 +82580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>71</v>
       </c>
@@ -82617,7 +82618,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>2756</v>
       </c>
@@ -82696,7 +82697,7 @@
         <v>-47</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>2919</v>
       </c>
@@ -82737,7 +82738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>873</v>
       </c>
@@ -82772,7 +82773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>3919</v>
       </c>
@@ -82932,7 +82933,7 @@
         <v>-73</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>3152</v>
       </c>
@@ -82973,7 +82974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>402</v>
       </c>
@@ -83014,7 +83015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>4512</v>
       </c>
@@ -83055,7 +83056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>3659</v>
       </c>
@@ -83096,7 +83097,7 @@
         <v>-72</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>1659</v>
       </c>
@@ -83137,7 +83138,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>768</v>
       </c>
@@ -83219,7 +83220,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>2849</v>
       </c>
@@ -83260,7 +83261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>2094</v>
       </c>
@@ -83301,7 +83302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>1633</v>
       </c>
@@ -83342,7 +83343,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>351</v>
       </c>
@@ -83380,7 +83381,7 @@
         <v>-72</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>4595</v>
       </c>
@@ -83421,7 +83422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>3343</v>
       </c>
@@ -83462,7 +83463,7 @@
         <v>-11</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>3246</v>
       </c>
@@ -83503,7 +83504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>406</v>
       </c>
@@ -83544,7 +83545,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>4053</v>
       </c>
@@ -83585,7 +83586,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>1627</v>
       </c>
@@ -83667,7 +83668,7 @@
         <v>-70</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>3924</v>
       </c>
@@ -83708,7 +83709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>4183</v>
       </c>
@@ -83749,7 +83750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>4299</v>
       </c>
@@ -83831,7 +83832,7 @@
         <v>-12</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>2927</v>
       </c>
@@ -83872,7 +83873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>2939</v>
       </c>
@@ -83911,7 +83912,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>1054</v>
       </c>
@@ -83952,7 +83953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>3694</v>
       </c>
@@ -83993,7 +83994,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>1775</v>
       </c>
@@ -84034,7 +84035,7 @@
         <v>-67</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>1378</v>
       </c>
@@ -84075,7 +84076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>3456</v>
       </c>
@@ -84116,7 +84117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>2787</v>
       </c>
@@ -84157,7 +84158,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>2132</v>
       </c>
@@ -84198,7 +84199,7 @@
         <v>-53</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>2564</v>
       </c>
@@ -84239,7 +84240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>823</v>
       </c>
@@ -84280,7 +84281,7 @@
         <v>-44</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>3093</v>
       </c>
@@ -84362,7 +84363,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>1216</v>
       </c>
@@ -84444,7 +84445,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>3946</v>
       </c>
@@ -84526,7 +84527,7 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>3040</v>
       </c>
@@ -84567,7 +84568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>2235</v>
       </c>
@@ -84608,7 +84609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>2632</v>
       </c>
@@ -84649,7 +84650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>556</v>
       </c>
@@ -84690,7 +84691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>1964</v>
       </c>
@@ -84731,7 +84732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>862</v>
       </c>
@@ -84772,7 +84773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>4125</v>
       </c>
@@ -84813,7 +84814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>3595</v>
       </c>
@@ -84854,7 +84855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>972</v>
       </c>
@@ -84895,7 +84896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>321</v>
       </c>
@@ -84936,7 +84937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>1229</v>
       </c>
@@ -84977,7 +84978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>597</v>
       </c>
@@ -85018,7 +85019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>3713</v>
       </c>
@@ -85059,7 +85060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>3583</v>
       </c>
@@ -85100,7 +85101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>3495</v>
       </c>
@@ -85141,7 +85142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>2135</v>
       </c>
@@ -85182,7 +85183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>4564</v>
       </c>
@@ -85223,7 +85224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>690</v>
       </c>
@@ -85264,7 +85265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>3874</v>
       </c>
@@ -85305,7 +85306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>793</v>
       </c>
@@ -85346,7 +85347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>1522</v>
       </c>
@@ -85592,7 +85593,7 @@
         <v>-15</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>2174</v>
       </c>
@@ -85633,7 +85634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>4508</v>
       </c>
@@ -85715,7 +85716,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>2012</v>
       </c>
@@ -85920,7 +85921,7 @@
         <v>-13</v>
       </c>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>981</v>
       </c>
@@ -85961,7 +85962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>97</v>
       </c>
@@ -85999,7 +86000,7 @@
         <v>-61</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>1572</v>
       </c>
@@ -86040,7 +86041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>1153</v>
       </c>
@@ -86081,7 +86082,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>2770</v>
       </c>
@@ -86160,7 +86161,7 @@
         <v>-9</v>
       </c>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>930</v>
       </c>
@@ -86201,7 +86202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>4592</v>
       </c>
@@ -86242,7 +86243,7 @@
         <v>-164</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>3590</v>
       </c>
@@ -86324,7 +86325,7 @@
         <v>-15</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>1624</v>
       </c>
@@ -86365,7 +86366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>3983</v>
       </c>
@@ -86406,7 +86407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>3488</v>
       </c>
@@ -86529,7 +86530,7 @@
         <v>-6</v>
       </c>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>4502</v>
       </c>
@@ -86611,7 +86612,7 @@
         <v>-8</v>
       </c>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>2772</v>
       </c>
@@ -86652,7 +86653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>2286</v>
       </c>
@@ -86728,7 +86729,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>804</v>
       </c>
@@ -86769,7 +86770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>669</v>
       </c>
@@ -86810,7 +86811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>1367</v>
       </c>
@@ -86851,7 +86852,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>1397</v>
       </c>
@@ -86892,7 +86893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>2897</v>
       </c>
@@ -86933,7 +86934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>1937</v>
       </c>
@@ -86974,7 +86975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>1961</v>
       </c>
@@ -87009,7 +87010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>75</v>
       </c>
@@ -87050,7 +87051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>487</v>
       </c>
@@ -87130,7 +87131,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>1304</v>
       </c>
@@ -87171,7 +87172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>1146</v>
       </c>
@@ -87212,7 +87213,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>449</v>
       </c>
@@ -87251,7 +87252,7 @@
         <v>-44</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>48</v>
       </c>
@@ -87292,7 +87293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>4104</v>
       </c>
@@ -87333,7 +87334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>2891</v>
       </c>
@@ -87374,7 +87375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>1267</v>
       </c>
@@ -87415,7 +87416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>1656</v>
       </c>
@@ -87456,7 +87457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>2250</v>
       </c>
@@ -87497,7 +87498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>3284</v>
       </c>
@@ -87538,7 +87539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>1241</v>
       </c>
@@ -87579,7 +87580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>2716</v>
       </c>
@@ -87620,7 +87621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>3189</v>
       </c>
@@ -87661,7 +87662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>666</v>
       </c>
@@ -87702,7 +87703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>2857</v>
       </c>
@@ -87743,7 +87744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>419</v>
       </c>
@@ -87825,7 +87826,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>2296</v>
       </c>
@@ -87866,7 +87867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>2526</v>
       </c>
@@ -87907,7 +87908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>1952</v>
       </c>
@@ -87946,7 +87947,7 @@
         <v>-107</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>3959</v>
       </c>
@@ -87987,7 +87988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>4058</v>
       </c>
@@ -88028,7 +88029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>1544</v>
       </c>
@@ -88069,7 +88070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>1577</v>
       </c>
@@ -88151,7 +88152,7 @@
         <v>-70</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>2548</v>
       </c>
@@ -88192,7 +88193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>3617</v>
       </c>
@@ -88233,7 +88234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>3559</v>
       </c>
@@ -88274,7 +88275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>3869</v>
       </c>
@@ -88315,7 +88316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>850</v>
       </c>
@@ -88356,7 +88357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>2707</v>
       </c>
@@ -88397,7 +88398,7 @@
         <v>-162</v>
       </c>
     </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>2540</v>
       </c>
@@ -88438,7 +88439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>950</v>
       </c>
@@ -88479,7 +88480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>2036</v>
       </c>
@@ -88520,7 +88521,7 @@
         <v>-110</v>
       </c>
     </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>1299</v>
       </c>
@@ -88643,7 +88644,7 @@
         <v>-51</v>
       </c>
     </row>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>3760</v>
       </c>
@@ -88684,7 +88685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>3172</v>
       </c>
@@ -88725,7 +88726,7 @@
         <v>-30</v>
       </c>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>3392</v>
       </c>
@@ -88766,7 +88767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>1405</v>
       </c>
@@ -88807,7 +88808,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>666</v>
       </c>
@@ -88889,7 +88890,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>3135</v>
       </c>
@@ -88930,7 +88931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>683</v>
       </c>
@@ -88971,7 +88972,7 @@
         <v>-45</v>
       </c>
     </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>3967</v>
       </c>
@@ -89012,7 +89013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>4185</v>
       </c>
@@ -89053,7 +89054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>2280</v>
       </c>
@@ -89094,7 +89095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>726</v>
       </c>
@@ -89136,12 +89137,95 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L247" xr:uid="{06520203-CDB0-4C4C-B268-5AFBB2D07120}"/>
+  <autoFilter ref="A1:L247" xr:uid="{06520203-CDB0-4C4C-B268-5AFBB2D07120}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="100"/>
+        <filter val="112"/>
+        <filter val="125"/>
+        <filter val="137"/>
+        <filter val="14"/>
+        <filter val="145"/>
+        <filter val="148"/>
+        <filter val="15"/>
+        <filter val="150"/>
+        <filter val="156"/>
+        <filter val="157"/>
+        <filter val="158"/>
+        <filter val="160"/>
+        <filter val="18"/>
+        <filter val="180"/>
+        <filter val="190"/>
+        <filter val="20"/>
+        <filter val="200"/>
+        <filter val="25"/>
+        <filter val="254"/>
+        <filter val="30"/>
+        <filter val="312"/>
+        <filter val="5"/>
+        <filter val="50"/>
+        <filter val="70"/>
+        <filter val="75"/>
+        <filter val="80"/>
+        <filter val="90"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="11">
+      <filters>
+        <filter val="-10"/>
+        <filter val="-100"/>
+        <filter val="-12"/>
+        <filter val="129"/>
+        <filter val="13"/>
+        <filter val="-13"/>
+        <filter val="-14"/>
+        <filter val="-15"/>
+        <filter val="-164"/>
+        <filter val="29"/>
+        <filter val="-3"/>
+        <filter val="-35"/>
+        <filter val="-47"/>
+        <filter val="48"/>
+        <filter val="-5"/>
+        <filter val="50"/>
+        <filter val="-51"/>
+        <filter val="52"/>
+        <filter val="-6"/>
+        <filter val="-7"/>
+        <filter val="-70"/>
+        <filter val="-73"/>
+        <filter val="-8"/>
+        <filter val="-86"/>
+        <filter val="9"/>
+        <filter val="-9"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A9D0198779F64D4583CB0D0F5191282D" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="265535fc1b2f34fa73935fce8401c032">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6a14bfa0-ee12-46b7-910d-7c55fe0c806e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="24633c4a450fef35b4745f60ee9eccd8" ns2:_="">
     <xsd:import namespace="6a14bfa0-ee12-46b7-910d-7c55fe0c806e"/>
@@ -89279,22 +89363,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86E2EAD6-3A6D-461A-BF09-23E6CBDBC756}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2BA5A7A-D550-4FF2-AB75-865AEB59BCF9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A031C75F-080B-4A14-9D1C-49C905405962}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -89310,21 +89396,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2BA5A7A-D550-4FF2-AB75-865AEB59BCF9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86E2EAD6-3A6D-461A-BF09-23E6CBDBC756}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>